<commit_message>
Fixed data-mapping issue in the raw data files. The update to quicR 3.0 messed up how the data was being associated in these files.
</commit_message>
<xml_diff>
--- a/raw/processedSamples/20250714_r9_GR_USDA-LNs_Nano-QuIC.xlsx
+++ b/raw/processedSamples/20250714_r9_GR_USDA-LNs_Nano-QuIC.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rowde002\Documents\Projects\usda-validation\raw\necropsy\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rowde002\Documents\Projects\usda-validation\raw\processedSamples\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FAEB9E8-0CDD-4468-9B84-4489264431DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2EDAFAC0-E17C-445D-9A70-14E64F67E376}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-14505" yWindow="105" windowWidth="14610" windowHeight="15585" xr2:uid="{AC565BB5-606A-427C-9BA9-84AB8C11ACE1}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{AC565BB5-606A-427C-9BA9-84AB8C11ACE1}"/>
   </bookViews>
   <sheets>
     <sheet name="Microplate Cycle 1 (0 h)" sheetId="2" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="563" uniqueCount="126">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="499" uniqueCount="118">
   <si>
     <t>User: USER</t>
   </si>
@@ -357,30 +357,6 @@
     <t>P</t>
   </si>
   <si>
-    <t>1944_RPLN</t>
-  </si>
-  <si>
-    <t>Y-18_RPLN</t>
-  </si>
-  <si>
-    <t>1905_RPLN</t>
-  </si>
-  <si>
-    <t>B-167_RPLN</t>
-  </si>
-  <si>
-    <t>B-227_RPLN</t>
-  </si>
-  <si>
-    <t>1904_RPLN</t>
-  </si>
-  <si>
-    <t>1943_RPLN</t>
-  </si>
-  <si>
-    <t>O-39_RPLN</t>
-  </si>
-  <si>
     <t>N</t>
   </si>
   <si>
@@ -646,7 +622,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -703,6 +679,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1086,7 +1065,7 @@
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.25">
       <c r="B14" t="s">
-        <v>114</v>
+        <v>106</v>
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.25">
@@ -1129,7 +1108,7 @@
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A16" s="10" t="s">
-        <v>115</v>
+        <v>107</v>
       </c>
       <c r="B16" s="11">
         <v>1352</v>
@@ -1164,7 +1143,7 @@
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A17" s="10" t="s">
-        <v>116</v>
+        <v>108</v>
       </c>
       <c r="B17" s="5">
         <v>1407</v>
@@ -1199,7 +1178,7 @@
     </row>
     <row r="18" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A18" s="10" t="s">
-        <v>117</v>
+        <v>109</v>
       </c>
       <c r="B18" s="5">
         <v>1442</v>
@@ -1234,7 +1213,7 @@
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A19" s="10" t="s">
-        <v>118</v>
+        <v>110</v>
       </c>
       <c r="B19" s="5">
         <v>1354</v>
@@ -1269,7 +1248,7 @@
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A20" s="10" t="s">
-        <v>119</v>
+        <v>111</v>
       </c>
       <c r="B20" s="5">
         <v>1394</v>
@@ -1304,7 +1283,7 @@
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A21" s="10" t="s">
-        <v>120</v>
+        <v>112</v>
       </c>
       <c r="B21" s="5">
         <v>1379</v>
@@ -1339,7 +1318,7 @@
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A22" s="10" t="s">
-        <v>121</v>
+        <v>113</v>
       </c>
       <c r="B22" s="5">
         <v>1338</v>
@@ -1374,7 +1353,7 @@
     </row>
     <row r="23" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A23" s="10" t="s">
-        <v>122</v>
+        <v>114</v>
       </c>
       <c r="B23" s="16">
         <v>1298</v>
@@ -1409,7 +1388,7 @@
     </row>
     <row r="25" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B25" t="s">
-        <v>123</v>
+        <v>115</v>
       </c>
       <c r="O25" s="19"/>
     </row>
@@ -1451,12 +1430,12 @@
         <v>12</v>
       </c>
       <c r="O26" s="20" t="s">
-        <v>124</v>
+        <v>116</v>
       </c>
     </row>
     <row r="27" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A27" s="10" t="s">
-        <v>115</v>
+        <v>107</v>
       </c>
       <c r="B27" s="11" t="s">
         <v>104</v>
@@ -1492,7 +1471,7 @@
     </row>
     <row r="28" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A28" s="10" t="s">
-        <v>116</v>
+        <v>108</v>
       </c>
       <c r="B28" s="5" t="s">
         <v>104</v>
@@ -1527,7 +1506,7 @@
     </row>
     <row r="29" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A29" s="10" t="s">
-        <v>117</v>
+        <v>109</v>
       </c>
       <c r="B29" s="5" t="s">
         <v>104</v>
@@ -1562,7 +1541,7 @@
     </row>
     <row r="30" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A30" s="10" t="s">
-        <v>118</v>
+        <v>110</v>
       </c>
       <c r="B30" s="5" t="s">
         <v>104</v>
@@ -1597,10 +1576,10 @@
     </row>
     <row r="31" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A31" s="10" t="s">
-        <v>119</v>
+        <v>111</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>113</v>
+        <v>105</v>
       </c>
       <c r="C31" s="12">
         <v>1978</v>
@@ -1632,10 +1611,10 @@
     </row>
     <row r="32" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A32" s="10" t="s">
-        <v>120</v>
+        <v>112</v>
       </c>
       <c r="B32" s="5" t="s">
-        <v>113</v>
+        <v>105</v>
       </c>
       <c r="C32" s="12">
         <v>1978</v>
@@ -1667,10 +1646,10 @@
     </row>
     <row r="33" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A33" s="10" t="s">
-        <v>121</v>
+        <v>113</v>
       </c>
       <c r="B33" s="5" t="s">
-        <v>113</v>
+        <v>105</v>
       </c>
       <c r="C33" s="12">
         <v>1978</v>
@@ -1702,10 +1681,10 @@
     </row>
     <row r="34" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A34" s="10" t="s">
-        <v>122</v>
+        <v>114</v>
       </c>
       <c r="B34" s="16" t="s">
-        <v>113</v>
+        <v>105</v>
       </c>
       <c r="C34" s="12">
         <v>1978</v>
@@ -1737,7 +1716,7 @@
     </row>
     <row r="36" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B36" t="s">
-        <v>125</v>
+        <v>117</v>
       </c>
       <c r="O36" s="19"/>
     </row>
@@ -1779,12 +1758,12 @@
         <v>12</v>
       </c>
       <c r="O37" s="20" t="s">
-        <v>124</v>
+        <v>116</v>
       </c>
     </row>
     <row r="38" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A38" s="10" t="s">
-        <v>115</v>
+        <v>107</v>
       </c>
       <c r="B38" s="11">
         <v>1000</v>
@@ -1820,7 +1799,7 @@
     </row>
     <row r="39" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A39" s="10" t="s">
-        <v>116</v>
+        <v>108</v>
       </c>
       <c r="B39" s="5">
         <v>1000</v>
@@ -1855,7 +1834,7 @@
     </row>
     <row r="40" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A40" s="10" t="s">
-        <v>117</v>
+        <v>109</v>
       </c>
       <c r="B40" s="5">
         <v>1000</v>
@@ -1890,7 +1869,7 @@
     </row>
     <row r="41" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A41" s="10" t="s">
-        <v>118</v>
+        <v>110</v>
       </c>
       <c r="B41" s="5">
         <v>1000</v>
@@ -1925,7 +1904,7 @@
     </row>
     <row r="42" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A42" s="10" t="s">
-        <v>119</v>
+        <v>111</v>
       </c>
       <c r="B42" s="5">
         <v>1000</v>
@@ -1960,7 +1939,7 @@
     </row>
     <row r="43" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A43" s="10" t="s">
-        <v>120</v>
+        <v>112</v>
       </c>
       <c r="B43" s="5">
         <v>1000</v>
@@ -1995,7 +1974,7 @@
     </row>
     <row r="44" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A44" s="10" t="s">
-        <v>121</v>
+        <v>113</v>
       </c>
       <c r="B44" s="5">
         <v>1000</v>
@@ -2030,7 +2009,7 @@
     </row>
     <row r="45" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A45" s="10" t="s">
-        <v>122</v>
+        <v>114</v>
       </c>
       <c r="B45" s="16">
         <v>1000</v>
@@ -67295,226 +67274,226 @@
         <v>6530</v>
       </c>
     </row>
-    <row r="302" spans="1:74" ht="30" x14ac:dyDescent="0.25">
-      <c r="A302" s="2" t="s">
+    <row r="302" spans="1:74" x14ac:dyDescent="0.25">
+      <c r="A302" s="22" t="s">
         <v>11</v>
       </c>
       <c r="B302" s="3"/>
-      <c r="C302" s="4" t="s">
+      <c r="C302" s="5" t="s">
         <v>104</v>
       </c>
-      <c r="D302" s="4" t="s">
+      <c r="D302" s="12">
+        <v>1978</v>
+      </c>
+      <c r="E302" s="12">
+        <v>1980</v>
+      </c>
+      <c r="F302" s="12">
+        <v>1981</v>
+      </c>
+      <c r="G302" s="12">
+        <v>2289</v>
+      </c>
+      <c r="H302" s="12">
+        <v>2290</v>
+      </c>
+      <c r="I302" s="12">
+        <v>2295</v>
+      </c>
+      <c r="J302" s="12">
+        <v>2291</v>
+      </c>
+      <c r="K302" s="12">
+        <v>2292</v>
+      </c>
+      <c r="L302" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="M302" s="12">
+        <v>1978</v>
+      </c>
+      <c r="N302" s="12">
+        <v>1980</v>
+      </c>
+      <c r="O302" s="12">
+        <v>1981</v>
+      </c>
+      <c r="P302" s="12">
+        <v>2289</v>
+      </c>
+      <c r="Q302" s="12">
+        <v>2290</v>
+      </c>
+      <c r="R302" s="12">
+        <v>2295</v>
+      </c>
+      <c r="S302" s="12">
+        <v>2291</v>
+      </c>
+      <c r="T302" s="12">
+        <v>2292</v>
+      </c>
+      <c r="U302" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="V302" s="12">
+        <v>1978</v>
+      </c>
+      <c r="W302" s="12">
+        <v>1980</v>
+      </c>
+      <c r="X302" s="12">
+        <v>1981</v>
+      </c>
+      <c r="Y302" s="12">
+        <v>2289</v>
+      </c>
+      <c r="Z302" s="12">
+        <v>2290</v>
+      </c>
+      <c r="AA302" s="12">
+        <v>2295</v>
+      </c>
+      <c r="AB302" s="12">
+        <v>2291</v>
+      </c>
+      <c r="AC302" s="12">
+        <v>2292</v>
+      </c>
+      <c r="AD302" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="AE302" s="12">
+        <v>1978</v>
+      </c>
+      <c r="AF302" s="12">
+        <v>1980</v>
+      </c>
+      <c r="AG302" s="12">
+        <v>1981</v>
+      </c>
+      <c r="AH302" s="12">
+        <v>2289</v>
+      </c>
+      <c r="AI302" s="12">
+        <v>2290</v>
+      </c>
+      <c r="AJ302" s="12">
+        <v>2295</v>
+      </c>
+      <c r="AK302" s="12">
+        <v>2291</v>
+      </c>
+      <c r="AL302" s="12">
+        <v>2292</v>
+      </c>
+      <c r="AM302" s="5" t="s">
         <v>105</v>
       </c>
-      <c r="E302" s="4" t="s">
-        <v>106</v>
-      </c>
-      <c r="F302" s="4" t="s">
-        <v>107</v>
-      </c>
-      <c r="G302" s="4" t="s">
-        <v>108</v>
-      </c>
-      <c r="H302" s="4" t="s">
-        <v>109</v>
-      </c>
-      <c r="I302" s="4" t="s">
-        <v>110</v>
-      </c>
-      <c r="J302" s="4" t="s">
-        <v>111</v>
-      </c>
-      <c r="K302" s="4" t="s">
-        <v>112</v>
-      </c>
-      <c r="L302" s="4" t="s">
-        <v>104</v>
-      </c>
-      <c r="M302" s="4" t="s">
+      <c r="AN302" s="12">
+        <v>1978</v>
+      </c>
+      <c r="AO302" s="12">
+        <v>1980</v>
+      </c>
+      <c r="AP302" s="12">
+        <v>1981</v>
+      </c>
+      <c r="AQ302" s="12">
+        <v>2289</v>
+      </c>
+      <c r="AR302" s="12">
+        <v>2290</v>
+      </c>
+      <c r="AS302" s="12">
+        <v>2295</v>
+      </c>
+      <c r="AT302" s="12">
+        <v>2291</v>
+      </c>
+      <c r="AU302" s="12">
+        <v>2292</v>
+      </c>
+      <c r="AV302" s="5" t="s">
         <v>105</v>
       </c>
-      <c r="N302" s="4" t="s">
-        <v>106</v>
-      </c>
-      <c r="O302" s="4" t="s">
-        <v>107</v>
-      </c>
-      <c r="P302" s="4" t="s">
-        <v>108</v>
-      </c>
-      <c r="Q302" s="4" t="s">
-        <v>109</v>
-      </c>
-      <c r="R302" s="4" t="s">
-        <v>110</v>
-      </c>
-      <c r="S302" s="4" t="s">
-        <v>111</v>
-      </c>
-      <c r="T302" s="4" t="s">
-        <v>112</v>
-      </c>
-      <c r="U302" s="4" t="s">
-        <v>104</v>
-      </c>
-      <c r="V302" s="4" t="s">
+      <c r="AW302" s="12">
+        <v>1978</v>
+      </c>
+      <c r="AX302" s="12">
+        <v>1980</v>
+      </c>
+      <c r="AY302" s="12">
+        <v>1981</v>
+      </c>
+      <c r="AZ302" s="12">
+        <v>2289</v>
+      </c>
+      <c r="BA302" s="12">
+        <v>2290</v>
+      </c>
+      <c r="BB302" s="12">
+        <v>2295</v>
+      </c>
+      <c r="BC302" s="12">
+        <v>2291</v>
+      </c>
+      <c r="BD302" s="12">
+        <v>2292</v>
+      </c>
+      <c r="BE302" s="5" t="s">
         <v>105</v>
       </c>
-      <c r="W302" s="4" t="s">
-        <v>106</v>
-      </c>
-      <c r="X302" s="4" t="s">
-        <v>107</v>
-      </c>
-      <c r="Y302" s="4" t="s">
-        <v>108</v>
-      </c>
-      <c r="Z302" s="4" t="s">
-        <v>109</v>
-      </c>
-      <c r="AA302" s="4" t="s">
-        <v>110</v>
-      </c>
-      <c r="AB302" s="4" t="s">
-        <v>111</v>
-      </c>
-      <c r="AC302" s="4" t="s">
-        <v>112</v>
-      </c>
-      <c r="AD302" s="4" t="s">
-        <v>104</v>
-      </c>
-      <c r="AE302" s="4" t="s">
+      <c r="BF302" s="12">
+        <v>1978</v>
+      </c>
+      <c r="BG302" s="12">
+        <v>1980</v>
+      </c>
+      <c r="BH302" s="12">
+        <v>1981</v>
+      </c>
+      <c r="BI302" s="12">
+        <v>2289</v>
+      </c>
+      <c r="BJ302" s="12">
+        <v>2290</v>
+      </c>
+      <c r="BK302" s="12">
+        <v>2295</v>
+      </c>
+      <c r="BL302" s="12">
+        <v>2291</v>
+      </c>
+      <c r="BM302" s="12">
+        <v>2292</v>
+      </c>
+      <c r="BN302" s="5" t="s">
         <v>105</v>
       </c>
-      <c r="AF302" s="4" t="s">
-        <v>106</v>
-      </c>
-      <c r="AG302" s="4" t="s">
-        <v>107</v>
-      </c>
-      <c r="AH302" s="4" t="s">
-        <v>108</v>
-      </c>
-      <c r="AI302" s="4" t="s">
-        <v>109</v>
-      </c>
-      <c r="AJ302" s="4" t="s">
-        <v>110</v>
-      </c>
-      <c r="AK302" s="4" t="s">
-        <v>111</v>
-      </c>
-      <c r="AL302" s="4" t="s">
-        <v>112</v>
-      </c>
-      <c r="AM302" s="4" t="s">
-        <v>113</v>
-      </c>
-      <c r="AN302" s="4" t="s">
-        <v>105</v>
-      </c>
-      <c r="AO302" s="4" t="s">
-        <v>106</v>
-      </c>
-      <c r="AP302" s="4" t="s">
-        <v>107</v>
-      </c>
-      <c r="AQ302" s="4" t="s">
-        <v>108</v>
-      </c>
-      <c r="AR302" s="4" t="s">
-        <v>109</v>
-      </c>
-      <c r="AS302" s="4" t="s">
-        <v>110</v>
-      </c>
-      <c r="AT302" s="4" t="s">
-        <v>111</v>
-      </c>
-      <c r="AU302" s="4" t="s">
-        <v>112</v>
-      </c>
-      <c r="AV302" s="4" t="s">
-        <v>113</v>
-      </c>
-      <c r="AW302" s="4" t="s">
-        <v>105</v>
-      </c>
-      <c r="AX302" s="4" t="s">
-        <v>106</v>
-      </c>
-      <c r="AY302" s="4" t="s">
-        <v>107</v>
-      </c>
-      <c r="AZ302" s="4" t="s">
-        <v>108</v>
-      </c>
-      <c r="BA302" s="4" t="s">
-        <v>109</v>
-      </c>
-      <c r="BB302" s="4" t="s">
-        <v>110</v>
-      </c>
-      <c r="BC302" s="4" t="s">
-        <v>111</v>
-      </c>
-      <c r="BD302" s="4" t="s">
-        <v>112</v>
-      </c>
-      <c r="BE302" s="4" t="s">
-        <v>113</v>
-      </c>
-      <c r="BF302" s="4" t="s">
-        <v>105</v>
-      </c>
-      <c r="BG302" s="4" t="s">
-        <v>106</v>
-      </c>
-      <c r="BH302" s="4" t="s">
-        <v>107</v>
-      </c>
-      <c r="BI302" s="4" t="s">
-        <v>108</v>
-      </c>
-      <c r="BJ302" s="4" t="s">
-        <v>109</v>
-      </c>
-      <c r="BK302" s="4" t="s">
-        <v>110</v>
-      </c>
-      <c r="BL302" s="4" t="s">
-        <v>111</v>
-      </c>
-      <c r="BM302" s="4" t="s">
-        <v>112</v>
-      </c>
-      <c r="BN302" s="4" t="s">
-        <v>113</v>
-      </c>
-      <c r="BO302" s="4" t="s">
-        <v>105</v>
-      </c>
-      <c r="BP302" s="4" t="s">
-        <v>106</v>
-      </c>
-      <c r="BQ302" s="4" t="s">
-        <v>107</v>
-      </c>
-      <c r="BR302" s="4" t="s">
-        <v>108</v>
-      </c>
-      <c r="BS302" s="4" t="s">
-        <v>109</v>
-      </c>
-      <c r="BT302" s="4" t="s">
-        <v>110</v>
-      </c>
-      <c r="BU302" s="4" t="s">
-        <v>111</v>
-      </c>
-      <c r="BV302" s="5" t="s">
-        <v>112</v>
+      <c r="BO302" s="12">
+        <v>1978</v>
+      </c>
+      <c r="BP302" s="12">
+        <v>1980</v>
+      </c>
+      <c r="BQ302" s="12">
+        <v>1981</v>
+      </c>
+      <c r="BR302" s="12">
+        <v>2289</v>
+      </c>
+      <c r="BS302" s="12">
+        <v>2290</v>
+      </c>
+      <c r="BT302" s="12">
+        <v>2295</v>
+      </c>
+      <c r="BU302" s="12">
+        <v>2291</v>
+      </c>
+      <c r="BV302" s="12">
+        <v>2292</v>
       </c>
     </row>
     <row r="303" spans="1:74" ht="30" x14ac:dyDescent="0.25">

</xml_diff>